<commit_message>
Lines of Effort tracker: house design language
Source workbook restyled by a repeatable script: red brand block with the
reversed logo in the masthead, pale title field and stat band, black
header row, priority chips in black / moawhango / pale, moawhango
progress bars, grid-grey rules, Army red kept for the stale warnings.
Data, formulas, validation, table and macro hooks unchanged; the
macro-enabled tracker rebuilt from it.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LgFPs3fMSncBgbYQ3PfA3o
</commit_message>
<xml_diff>
--- a/assets/lines-of-effort-tracker.xlsx
+++ b/assets/lines-of-effort-tracker.xlsx
@@ -42,7 +42,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="73">
   <si>
-    <t>NZALC HQ - LINES OF EFFORT TRACKER</t>
+    <t>NZALC HQ Lines of Effort Tracker</t>
   </si>
   <si>
     <t>ACTIVE LINES OF EFFORT</t>
@@ -283,27 +283,27 @@
     <font>
       <b/>
       <sz val="16"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="8"/>
-      <color rgb="FF222222"/>
+      <sz val="7"/>
+      <color rgb="FF002516"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="24"/>
-      <color rgb="FF222222"/>
+      <sz val="22"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <sz val="8.5"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -316,7 +316,7 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="0" tint="-0.14999847407452621"/>
+      <color rgb="FF8A8A8A"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -349,7 +349,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FFF6F6F3"/>
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
@@ -364,16 +364,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFD9D9D9"/>
+        <color rgb="FFD9D9D2"/>
       </left>
       <right style="thin">
-        <color rgb="FFD9D9D9"/>
+        <color rgb="FFD9D9D2"/>
       </right>
       <top style="thin">
-        <color rgb="FFD9D9D9"/>
+        <color rgb="FFD9D9D2"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
+        <color rgb="FFD9D9D2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -419,7 +419,7 @@
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -437,7 +437,7 @@
       <font>
         <b/>
         <sz val="10"/>
-        <color rgb="FFC98A00"/>
+        <color rgb="FFC62026"/>
         <name val="Arial"/>
         <charset val="1"/>
       </font>
@@ -445,8 +445,8 @@
     <dxf>
       <font>
         <b/>
-        <sz val="24"/>
-        <color rgb="FFC98A00"/>
+        <sz val="22"/>
+        <color rgb="FFC62026"/>
         <name val="Arial"/>
         <charset val="1"/>
       </font>
@@ -455,13 +455,13 @@
       <font>
         <b/>
         <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FF222222"/>
         <name val="Arial"/>
         <charset val="1"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FF2E7D32"/>
+          <bgColor rgb="FFEEF1E5"/>
         </patternFill>
       </fill>
     </dxf>
@@ -469,13 +469,13 @@
       <font>
         <b/>
         <sz val="10"/>
-        <color rgb="FF3A2B00"/>
+        <color rgb="FF002516"/>
         <name val="Arial"/>
         <charset val="1"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC98A00"/>
+          <bgColor rgb="FFCDD2B7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -489,7 +489,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC0392B"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -572,6 +572,44 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1219200" cy="406400"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="NZ Army"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1219200" cy="406400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -775,7 +813,7 @@
   <dimension ref="A1:G31"/>
   <sheetFormatPr defaultColWidth="8.609375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.390625" customWidth="1"/>
+    <col min="1" max="1" width="18.5" customWidth="1"/>
     <col min="2" max="2" width="41.96875" customWidth="1"/>
     <col min="3" max="3" width="39.81640625" customWidth="1"/>
     <col min="4" max="4" width="32.8203125" customWidth="1"/>
@@ -785,11 +823,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+    <row r="2" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="13"/>
+      <c r="B2" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="13"/>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
       <c r="E2" s="13"/>
@@ -1342,7 +1380,7 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="B2:G2"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="A5:B5"/>
@@ -1364,7 +1402,7 @@
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
-        <color rgb="FF9DBE85"/>
+        <color rgb="FFCDD2B7"/>
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
@@ -1399,6 +1437,7 @@
     <oddHeader>&amp;C&amp;"Calibri Bold"&amp;12&amp;K000000 UNCLASSIFIED&amp;1#_x000D_</oddHeader>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri Bold"&amp;12&amp;K000000 UNCLASSIFIED</oddFooter>
   </headerFooter>
+  <drawing r:id="rIdDrawing"/>
   <tableParts count="1">
     <tablePart r:id="rId2"/>
   </tableParts>
@@ -1414,7 +1453,7 @@
               <x14:cfvo type="num">
                 <xm:f>1</xm:f>
               </x14:cfvo>
-              <x14:negativeFillColor rgb="FF9DBE85"/>
+              <x14:negativeFillColor rgb="FFCDD2B7"/>
             </x14:dataBar>
           </x14:cfRule>
           <xm:sqref>D8:D38</xm:sqref>

</xml_diff>